<commit_message>
update excel file shape
</commit_message>
<xml_diff>
--- a/IT23620148.xlsx
+++ b/IT23620148.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\test_automation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\IT23620148\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C274AAB-4BF6-4319-ACD5-C70EC86931A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{291DE534-6CA4-488B-95F1-B887D90D1BCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="722" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -946,7 +946,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -969,12 +969,108 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -988,13 +1084,6 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1004,8 +1093,48 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1411,6 +1540,36 @@
       </border>
     </dxf>
     <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -1435,36 +1594,6 @@
       </fill>
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1479,7 +1608,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{87841D95-ECE1-4830-8D7A-436E086575CA}" name="Table1" displayName="Table1" ref="A1:H51" totalsRowShown="0" headerRowDxfId="0" dataDxfId="9" headerRowBorderDxfId="11" tableBorderDxfId="12" totalsRowBorderDxfId="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{87841D95-ECE1-4830-8D7A-436E086575CA}" name="Table1" displayName="Table1" ref="A1:H51" totalsRowShown="0" headerRowDxfId="0" dataDxfId="12" headerRowBorderDxfId="10" tableBorderDxfId="11" totalsRowBorderDxfId="9">
   <autoFilter ref="A1:H51" xr:uid="{87841D95-ECE1-4830-8D7A-436E086575CA}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{08B07A38-FC26-4573-8924-F66BBCD7BB62}" name="Test Case ID" dataDxfId="8"/>
@@ -1761,47 +1890,47 @@
   <dimension ref="A1:H51"/>
   <sheetFormatPr defaultRowHeight="49.95" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.88671875" style="5" customWidth="1"/>
-    <col min="2" max="2" width="13.6640625" style="5" customWidth="1"/>
-    <col min="3" max="3" width="22.109375" style="5" customWidth="1"/>
-    <col min="4" max="4" width="25.33203125" style="5" customWidth="1"/>
-    <col min="5" max="5" width="22.5546875" style="5" customWidth="1"/>
-    <col min="6" max="6" width="8.88671875" style="10" customWidth="1"/>
-    <col min="7" max="7" width="22.21875" style="5" customWidth="1"/>
-    <col min="8" max="8" width="16" style="5" customWidth="1"/>
-    <col min="9" max="10" width="12.33203125" style="5" customWidth="1"/>
-    <col min="11" max="15" width="8.88671875" style="5" customWidth="1"/>
-    <col min="16" max="16384" width="8.88671875" style="5"/>
+    <col min="1" max="1" width="10.88671875" style="8" customWidth="1"/>
+    <col min="2" max="2" width="13.6640625" style="8" customWidth="1"/>
+    <col min="3" max="3" width="22.109375" style="8" customWidth="1"/>
+    <col min="4" max="4" width="25.33203125" style="8" customWidth="1"/>
+    <col min="5" max="5" width="22.5546875" style="8" customWidth="1"/>
+    <col min="6" max="6" width="8.88671875" style="9" customWidth="1"/>
+    <col min="7" max="7" width="22.21875" style="8" customWidth="1"/>
+    <col min="8" max="8" width="16" style="8" customWidth="1"/>
+    <col min="9" max="10" width="12.33203125" style="8" customWidth="1"/>
+    <col min="11" max="15" width="8.88671875" style="8" customWidth="1"/>
+    <col min="16" max="16384" width="8.88671875" style="8"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="36.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="11" t="s">
         <v>210</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="13" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="14" t="s">
         <v>6</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -1816,18 +1945,18 @@
       <c r="E2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="G2" s="9" t="s">
+      <c r="F2" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" s="6" t="s">
         <v>264</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="15" t="s">
         <v>213</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="14" t="s">
         <v>12</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -1842,18 +1971,18 @@
       <c r="E3" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="F3" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G3" s="9" t="s">
+      <c r="F3" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" s="6" t="s">
         <v>264</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" s="15" t="s">
         <v>214</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="14" t="s">
         <v>17</v>
       </c>
       <c r="B4" s="1" t="s">
@@ -1868,18 +1997,18 @@
       <c r="E4" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="F4" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G4" s="9" t="s">
+      <c r="F4" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" s="6" t="s">
         <v>265</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="H4" s="15" t="s">
         <v>215</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="14" t="s">
         <v>21</v>
       </c>
       <c r="B5" s="1" t="s">
@@ -1894,18 +2023,18 @@
       <c r="E5" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="F5" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G5" s="9" t="s">
+      <c r="F5" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" s="6" t="s">
         <v>265</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="H5" s="15" t="s">
         <v>216</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="14" t="s">
         <v>25</v>
       </c>
       <c r="B6" s="1" t="s">
@@ -1920,18 +2049,18 @@
       <c r="E6" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="F6" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="G6" s="9" t="s">
+      <c r="F6" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" s="6" t="s">
         <v>266</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="H6" s="15" t="s">
         <v>217</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="14" t="s">
         <v>29</v>
       </c>
       <c r="B7" s="1" t="s">
@@ -1946,18 +2075,18 @@
       <c r="E7" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="F7" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G7" s="9" t="s">
+      <c r="F7" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G7" s="6" t="s">
         <v>266</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="H7" s="15" t="s">
         <v>218</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="14" t="s">
         <v>33</v>
       </c>
       <c r="B8" s="1" t="s">
@@ -1972,18 +2101,18 @@
       <c r="E8" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="F8" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G8" s="9" t="s">
+      <c r="F8" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" s="6" t="s">
         <v>267</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="H8" s="15" t="s">
         <v>219</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="14" t="s">
         <v>37</v>
       </c>
       <c r="B9" s="1" t="s">
@@ -1998,18 +2127,18 @@
       <c r="E9" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F9" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G9" s="9" t="s">
+      <c r="F9" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G9" s="6" t="s">
         <v>267</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="H9" s="15" t="s">
         <v>220</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
+      <c r="A10" s="14" t="s">
         <v>41</v>
       </c>
       <c r="B10" s="1" t="s">
@@ -2024,18 +2153,18 @@
       <c r="E10" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="F10" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G10" s="9" t="s">
+      <c r="F10" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G10" s="6" t="s">
         <v>268</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="H10" s="15" t="s">
         <v>221</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="1" t="s">
+      <c r="A11" s="14" t="s">
         <v>45</v>
       </c>
       <c r="B11" s="1" t="s">
@@ -2050,18 +2179,18 @@
       <c r="E11" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="F11" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G11" s="9" t="s">
+      <c r="F11" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G11" s="6" t="s">
         <v>268</v>
       </c>
-      <c r="H11" s="2" t="s">
+      <c r="H11" s="15" t="s">
         <v>222</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="1" t="s">
+      <c r="A12" s="14" t="s">
         <v>49</v>
       </c>
       <c r="B12" s="1" t="s">
@@ -2076,18 +2205,18 @@
       <c r="E12" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="F12" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G12" s="9" t="s">
+      <c r="F12" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G12" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="H12" s="2" t="s">
+      <c r="H12" s="15" t="s">
         <v>223</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="1" t="s">
+      <c r="A13" s="14" t="s">
         <v>53</v>
       </c>
       <c r="B13" s="1" t="s">
@@ -2102,18 +2231,18 @@
       <c r="E13" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="F13" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G13" s="9" t="s">
+      <c r="F13" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G13" s="6" t="s">
         <v>269</v>
       </c>
-      <c r="H13" s="2" t="s">
+      <c r="H13" s="15" t="s">
         <v>224</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="1" t="s">
+      <c r="A14" s="14" t="s">
         <v>57</v>
       </c>
       <c r="B14" s="1" t="s">
@@ -2128,18 +2257,18 @@
       <c r="E14" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="F14" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G14" s="9" t="s">
+      <c r="F14" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G14" s="6" t="s">
         <v>270</v>
       </c>
-      <c r="H14" s="2" t="s">
+      <c r="H14" s="15" t="s">
         <v>225</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="1" t="s">
+      <c r="A15" s="14" t="s">
         <v>61</v>
       </c>
       <c r="B15" s="1" t="s">
@@ -2154,18 +2283,18 @@
       <c r="E15" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="F15" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G15" s="9" t="s">
+      <c r="F15" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G15" s="6" t="s">
         <v>270</v>
       </c>
-      <c r="H15" s="2" t="s">
+      <c r="H15" s="15" t="s">
         <v>226</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="1" t="s">
+      <c r="A16" s="14" t="s">
         <v>65</v>
       </c>
       <c r="B16" s="1" t="s">
@@ -2180,18 +2309,18 @@
       <c r="E16" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="F16" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G16" s="9" t="s">
+      <c r="F16" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G16" s="6" t="s">
         <v>271</v>
       </c>
-      <c r="H16" s="2" t="s">
+      <c r="H16" s="15" t="s">
         <v>227</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="1" t="s">
+      <c r="A17" s="14" t="s">
         <v>69</v>
       </c>
       <c r="B17" s="1" t="s">
@@ -2206,18 +2335,18 @@
       <c r="E17" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="F17" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G17" s="9" t="s">
+      <c r="F17" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G17" s="6" t="s">
         <v>271</v>
       </c>
-      <c r="H17" s="2" t="s">
+      <c r="H17" s="15" t="s">
         <v>228</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="1" t="s">
+      <c r="A18" s="14" t="s">
         <v>73</v>
       </c>
       <c r="B18" s="1" t="s">
@@ -2232,18 +2361,18 @@
       <c r="E18" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="F18" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G18" s="9" t="s">
+      <c r="F18" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G18" s="6" t="s">
         <v>272</v>
       </c>
-      <c r="H18" s="2" t="s">
+      <c r="H18" s="15" t="s">
         <v>229</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="1" t="s">
+      <c r="A19" s="14" t="s">
         <v>77</v>
       </c>
       <c r="B19" s="1" t="s">
@@ -2258,18 +2387,18 @@
       <c r="E19" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="F19" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G19" s="9" t="s">
+      <c r="F19" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G19" s="6" t="s">
         <v>272</v>
       </c>
-      <c r="H19" s="2" t="s">
+      <c r="H19" s="15" t="s">
         <v>230</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="1" t="s">
+      <c r="A20" s="14" t="s">
         <v>81</v>
       </c>
       <c r="B20" s="1" t="s">
@@ -2284,18 +2413,18 @@
       <c r="E20" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="F20" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G20" s="9" t="s">
+      <c r="F20" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G20" s="6" t="s">
         <v>273</v>
       </c>
-      <c r="H20" s="2" t="s">
+      <c r="H20" s="15" t="s">
         <v>231</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="1" t="s">
+      <c r="A21" s="14" t="s">
         <v>85</v>
       </c>
       <c r="B21" s="1" t="s">
@@ -2310,18 +2439,18 @@
       <c r="E21" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="F21" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G21" s="9" t="s">
+      <c r="F21" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G21" s="6" t="s">
         <v>273</v>
       </c>
-      <c r="H21" s="2" t="s">
+      <c r="H21" s="15" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="1" t="s">
+      <c r="A22" s="14" t="s">
         <v>89</v>
       </c>
       <c r="B22" s="1" t="s">
@@ -2336,18 +2465,18 @@
       <c r="E22" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="F22" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G22" s="9" t="s">
+      <c r="F22" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G22" s="6" t="s">
         <v>274</v>
       </c>
-      <c r="H22" s="2" t="s">
+      <c r="H22" s="15" t="s">
         <v>233</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="1" t="s">
+      <c r="A23" s="14" t="s">
         <v>93</v>
       </c>
       <c r="B23" s="1" t="s">
@@ -2362,18 +2491,18 @@
       <c r="E23" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="F23" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G23" s="9" t="s">
+      <c r="F23" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G23" s="6" t="s">
         <v>275</v>
       </c>
-      <c r="H23" s="2" t="s">
+      <c r="H23" s="15" t="s">
         <v>234</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="1" t="s">
+      <c r="A24" s="14" t="s">
         <v>97</v>
       </c>
       <c r="B24" s="1" t="s">
@@ -2388,18 +2517,18 @@
       <c r="E24" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="F24" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G24" s="9" t="s">
+      <c r="F24" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G24" s="6" t="s">
         <v>276</v>
       </c>
-      <c r="H24" s="2" t="s">
+      <c r="H24" s="15" t="s">
         <v>235</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="1" t="s">
+      <c r="A25" s="14" t="s">
         <v>101</v>
       </c>
       <c r="B25" s="1" t="s">
@@ -2414,18 +2543,18 @@
       <c r="E25" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="F25" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G25" s="9" t="s">
+      <c r="F25" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G25" s="6" t="s">
         <v>276</v>
       </c>
-      <c r="H25" s="2" t="s">
+      <c r="H25" s="15" t="s">
         <v>236</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="1" t="s">
+      <c r="A26" s="14" t="s">
         <v>105</v>
       </c>
       <c r="B26" s="1" t="s">
@@ -2440,18 +2569,18 @@
       <c r="E26" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="F26" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G26" s="9" t="s">
+      <c r="F26" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G26" s="6" t="s">
         <v>277</v>
       </c>
-      <c r="H26" s="2" t="s">
+      <c r="H26" s="15" t="s">
         <v>237</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="1" t="s">
+      <c r="A27" s="14" t="s">
         <v>109</v>
       </c>
       <c r="B27" s="1" t="s">
@@ -2466,18 +2595,18 @@
       <c r="E27" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="F27" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G27" s="9" t="s">
+      <c r="F27" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G27" s="6" t="s">
         <v>277</v>
       </c>
-      <c r="H27" s="2" t="s">
+      <c r="H27" s="15" t="s">
         <v>238</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="1" t="s">
+      <c r="A28" s="14" t="s">
         <v>113</v>
       </c>
       <c r="B28" s="1" t="s">
@@ -2492,18 +2621,18 @@
       <c r="E28" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="F28" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G28" s="9" t="s">
+      <c r="F28" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G28" s="6" t="s">
         <v>278</v>
       </c>
-      <c r="H28" s="11" t="s">
+      <c r="H28" s="16" t="s">
         <v>239</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="1" t="s">
+      <c r="A29" s="14" t="s">
         <v>117</v>
       </c>
       <c r="B29" s="1" t="s">
@@ -2518,18 +2647,18 @@
       <c r="E29" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="F29" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G29" s="9" t="s">
+      <c r="F29" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G29" s="6" t="s">
         <v>274</v>
       </c>
-      <c r="H29" s="2" t="s">
+      <c r="H29" s="15" t="s">
         <v>240</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="1" t="s">
+      <c r="A30" s="14" t="s">
         <v>121</v>
       </c>
       <c r="B30" s="1" t="s">
@@ -2544,18 +2673,18 @@
       <c r="E30" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="F30" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G30" s="9" t="s">
+      <c r="F30" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G30" s="6" t="s">
         <v>275</v>
       </c>
-      <c r="H30" s="2" t="s">
+      <c r="H30" s="15" t="s">
         <v>241</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="1" t="s">
+      <c r="A31" s="14" t="s">
         <v>125</v>
       </c>
       <c r="B31" s="1" t="s">
@@ -2570,22 +2699,22 @@
       <c r="E31" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="F31" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G31" s="9" t="s">
+      <c r="F31" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G31" s="6" t="s">
         <v>275</v>
       </c>
-      <c r="H31" s="2" t="s">
+      <c r="H31" s="15" t="s">
         <v>242</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="1" t="s">
+      <c r="A32" s="14" t="s">
         <v>129</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>130</v>
@@ -2596,18 +2725,18 @@
       <c r="E32" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="F32" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G32" s="9" t="s">
+      <c r="F32" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G32" s="6" t="s">
         <v>279</v>
       </c>
-      <c r="H32" s="2" t="s">
+      <c r="H32" s="15" t="s">
         <v>243</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="1" t="s">
+      <c r="A33" s="14" t="s">
         <v>133</v>
       </c>
       <c r="B33" s="1" t="s">
@@ -2622,22 +2751,22 @@
       <c r="E33" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="F33" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G33" s="9" t="s">
+      <c r="F33" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G33" s="6" t="s">
         <v>279</v>
       </c>
-      <c r="H33" s="2" t="s">
+      <c r="H33" s="15" t="s">
         <v>244</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="1" t="s">
+      <c r="A34" s="14" t="s">
         <v>137</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>138</v>
@@ -2648,22 +2777,22 @@
       <c r="E34" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="F34" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G34" s="9" t="s">
+      <c r="F34" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G34" s="6" t="s">
         <v>280</v>
       </c>
-      <c r="H34" s="2" t="s">
+      <c r="H34" s="15" t="s">
         <v>245</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="1" t="s">
+      <c r="A35" s="14" t="s">
         <v>141</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>142</v>
@@ -2674,18 +2803,18 @@
       <c r="E35" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="F35" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G35" s="9" t="s">
+      <c r="F35" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G35" s="6" t="s">
         <v>278</v>
       </c>
-      <c r="H35" s="2" t="s">
+      <c r="H35" s="15" t="s">
         <v>246</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="1" t="s">
+      <c r="A36" s="14" t="s">
         <v>145</v>
       </c>
       <c r="B36" s="1" t="s">
@@ -2700,18 +2829,18 @@
       <c r="E36" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="F36" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G36" s="9" t="s">
+      <c r="F36" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G36" s="6" t="s">
         <v>281</v>
       </c>
-      <c r="H36" s="2" t="s">
+      <c r="H36" s="15" t="s">
         <v>247</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="1" t="s">
+      <c r="A37" s="14" t="s">
         <v>149</v>
       </c>
       <c r="B37" s="1" t="s">
@@ -2726,22 +2855,22 @@
       <c r="E37" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="F37" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G37" s="9" t="s">
+      <c r="F37" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G37" s="6" t="s">
         <v>281</v>
       </c>
-      <c r="H37" s="2" t="s">
+      <c r="H37" s="15" t="s">
         <v>248</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="1" t="s">
+      <c r="A38" s="14" t="s">
         <v>153</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>154</v>
@@ -2752,18 +2881,18 @@
       <c r="E38" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="F38" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G38" s="9" t="s">
+      <c r="F38" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G38" s="6" t="s">
         <v>282</v>
       </c>
-      <c r="H38" s="2" t="s">
+      <c r="H38" s="15" t="s">
         <v>249</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="1" t="s">
+      <c r="A39" s="14" t="s">
         <v>157</v>
       </c>
       <c r="B39" s="1" t="s">
@@ -2778,22 +2907,22 @@
       <c r="E39" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="F39" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G39" s="9" t="s">
+      <c r="F39" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G39" s="6" t="s">
         <v>282</v>
       </c>
-      <c r="H39" s="2" t="s">
+      <c r="H39" s="15" t="s">
         <v>250</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="1" t="s">
+      <c r="A40" s="14" t="s">
         <v>161</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>162</v>
@@ -2804,18 +2933,18 @@
       <c r="E40" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="F40" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G40" s="9" t="s">
+      <c r="F40" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G40" s="6" t="s">
         <v>283</v>
       </c>
-      <c r="H40" s="2" t="s">
+      <c r="H40" s="15" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="41" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="1" t="s">
+      <c r="A41" s="14" t="s">
         <v>165</v>
       </c>
       <c r="B41" s="1" t="s">
@@ -2830,22 +2959,22 @@
       <c r="E41" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="F41" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G41" s="9" t="s">
+      <c r="F41" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G41" s="6" t="s">
         <v>283</v>
       </c>
-      <c r="H41" s="2" t="s">
+      <c r="H41" s="15" t="s">
         <v>252</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="1" t="s">
+      <c r="A42" s="14" t="s">
         <v>169</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>170</v>
@@ -2856,18 +2985,18 @@
       <c r="E42" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="F42" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G42" s="9" t="s">
+      <c r="F42" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G42" s="6" t="s">
         <v>284</v>
       </c>
-      <c r="H42" s="2" t="s">
+      <c r="H42" s="15" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="1" t="s">
+      <c r="A43" s="14" t="s">
         <v>173</v>
       </c>
       <c r="B43" s="1" t="s">
@@ -2882,22 +3011,22 @@
       <c r="E43" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="F43" s="10" t="s">
+      <c r="F43" s="7" t="s">
         <v>11</v>
       </c>
       <c r="G43" s="3" t="s">
         <v>284</v>
       </c>
-      <c r="H43" s="2" t="s">
+      <c r="H43" s="15" t="s">
         <v>254</v>
       </c>
     </row>
     <row r="44" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="1" t="s">
+      <c r="A44" s="14" t="s">
         <v>177</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="C44" s="2" t="s">
         <v>178</v>
@@ -2908,18 +3037,18 @@
       <c r="E44" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="F44" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G44" s="9" t="s">
+      <c r="F44" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G44" s="6" t="s">
         <v>285</v>
       </c>
-      <c r="H44" s="2" t="s">
+      <c r="H44" s="15" t="s">
         <v>255</v>
       </c>
     </row>
     <row r="45" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="1" t="s">
+      <c r="A45" s="14" t="s">
         <v>181</v>
       </c>
       <c r="B45" s="1" t="s">
@@ -2934,22 +3063,22 @@
       <c r="E45" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="F45" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G45" s="9" t="s">
+      <c r="F45" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G45" s="6" t="s">
         <v>285</v>
       </c>
-      <c r="H45" s="2" t="s">
+      <c r="H45" s="15" t="s">
         <v>256</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="1" t="s">
+      <c r="A46" s="14" t="s">
         <v>185</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="C46" s="4" t="s">
         <v>186</v>
@@ -2960,18 +3089,18 @@
       <c r="E46" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="F46" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G46" s="9" t="s">
+      <c r="F46" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G46" s="6" t="s">
         <v>286</v>
       </c>
-      <c r="H46" s="2" t="s">
+      <c r="H46" s="15" t="s">
         <v>257</v>
       </c>
     </row>
     <row r="47" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="1" t="s">
+      <c r="A47" s="14" t="s">
         <v>189</v>
       </c>
       <c r="B47" s="1" t="s">
@@ -2986,22 +3115,22 @@
       <c r="E47" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="F47" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G47" s="9" t="s">
+      <c r="F47" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G47" s="6" t="s">
         <v>286</v>
       </c>
-      <c r="H47" s="2" t="s">
+      <c r="H47" s="15" t="s">
         <v>258</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="1" t="s">
+      <c r="A48" s="14" t="s">
         <v>193</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="C48" s="2" t="s">
         <v>194</v>
@@ -3012,18 +3141,18 @@
       <c r="E48" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="F48" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G48" s="9" t="s">
+      <c r="F48" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G48" s="6" t="s">
         <v>287</v>
       </c>
-      <c r="H48" s="2" t="s">
+      <c r="H48" s="15" t="s">
         <v>259</v>
       </c>
     </row>
     <row r="49" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="1" t="s">
+      <c r="A49" s="14" t="s">
         <v>197</v>
       </c>
       <c r="B49" s="1" t="s">
@@ -3038,18 +3167,18 @@
       <c r="E49" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="F49" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G49" s="9" t="s">
+      <c r="F49" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G49" s="6" t="s">
         <v>287</v>
       </c>
-      <c r="H49" s="2" t="s">
+      <c r="H49" s="15" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="50" spans="1:8" ht="70.8" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="1" t="s">
+      <c r="A50" s="14" t="s">
         <v>201</v>
       </c>
       <c r="B50" s="1" t="s">
@@ -3064,39 +3193,39 @@
       <c r="E50" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="F50" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G50" s="9" t="s">
+      <c r="F50" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G50" s="6" t="s">
         <v>263</v>
       </c>
-      <c r="H50" s="2" t="s">
+      <c r="H50" s="15" t="s">
         <v>261</v>
       </c>
     </row>
     <row r="51" spans="1:8" ht="72.599999999999994" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="1" t="s">
+      <c r="A51" s="17" t="s">
         <v>206</v>
       </c>
-      <c r="B51" s="1" t="s">
+      <c r="B51" s="18" t="s">
         <v>202</v>
       </c>
-      <c r="C51" s="2" t="s">
+      <c r="C51" s="19" t="s">
         <v>207</v>
       </c>
-      <c r="D51" s="2" t="s">
+      <c r="D51" s="19" t="s">
         <v>208</v>
       </c>
-      <c r="E51" s="2" t="s">
+      <c r="E51" s="19" t="s">
         <v>209</v>
       </c>
-      <c r="F51" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G51" s="9" t="s">
+      <c r="F51" s="20" t="s">
+        <v>11</v>
+      </c>
+      <c r="G51" s="21" t="s">
         <v>263</v>
       </c>
-      <c r="H51" s="2" t="s">
+      <c r="H51" s="22" t="s">
         <v>262</v>
       </c>
     </row>

</xml_diff>